<commit_message>
Se adjunta el MDJ de Diagramas de Caso de Uso y sus PNG, junto a la Planilla actualizada.
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Proyecto/Planilla_Requerimientos_Final.xlsx
+++ b/Fase 1/Evidencias Proyecto/Planilla_Requerimientos_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h8_hate machine\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h8_hate machine\Documents\GitHub\Sistema Web de Tarificación Telefónica\Fase 1\Evidencias Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00578E2-C036-4B1D-8C94-58014B10212F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDFC4B3-EE8F-4406-B49B-26BE6934E375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="228">
   <si>
     <t>[Nombre del Requerimiento]</t>
   </si>
@@ -229,9 +229,6 @@
   </si>
   <si>
     <t>Sistema Web, Desarrollador, Usuario , Base de Datos</t>
-  </si>
-  <si>
-    <t>Sistema Web, Desarrollador</t>
   </si>
   <si>
     <t>Sistema Web, Base de Datos</t>
@@ -808,6 +805,28 @@
     <t>Indica los actores que interactúan o se ven involucrados en el requerimiento.
 Estos pueden incluir: Empleado, Administrador, Sistema Web
 Base de Datos, API ,y Desarrollador</t>
+  </si>
+  <si>
+    <t>Permite al Administrador modificar los datos de cuenta de una cuenta Empleado</t>
+  </si>
+  <si>
+    <t>Administrador, Empleado, 
+Sistema Web, Base de Datos</t>
+  </si>
+  <si>
+    <t>Sistema Web, Base de Datos, Administrador,
+Empleado</t>
+  </si>
+  <si>
+    <t>Administrador, Sistema Web, Empleado
+Base de Datos</t>
+  </si>
+  <si>
+    <t>Sistema Web, Base de Datos, Empleado,
+Administrador</t>
+  </si>
+  <si>
+    <t>Sistema Web, Desarrollador, Empleado, Administrador</t>
   </si>
 </sst>
 </file>
@@ -1056,7 +1075,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1247,6 +1266,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1548,7 +1570,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
@@ -1556,7 +1578,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1564,7 +1586,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="56.25" x14ac:dyDescent="0.25">
@@ -1572,7 +1594,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1580,7 +1602,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1588,7 +1610,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
@@ -1596,7 +1618,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1616,7 +1638,7 @@
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="47" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.5703125" customWidth="1"/>
-    <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="82.28515625" customWidth="1"/>
     <col min="6" max="6" width="74.85546875" customWidth="1"/>
     <col min="7" max="7" width="13.140625" customWidth="1"/>
@@ -1656,16 +1678,16 @@
         <v>57</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="57" t="s">
-        <v>68</v>
+        <v>186</v>
+      </c>
+      <c r="D2" s="71" t="s">
+        <v>224</v>
       </c>
       <c r="E2" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>170</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>171</v>
       </c>
       <c r="G2" s="20" t="s">
         <v>12</v>
@@ -1679,16 +1701,16 @@
         <v>61</v>
       </c>
       <c r="C3" s="58" t="s">
-        <v>184</v>
-      </c>
-      <c r="D3" s="57" t="s">
-        <v>68</v>
+        <v>183</v>
+      </c>
+      <c r="D3" s="71" t="s">
+        <v>226</v>
       </c>
       <c r="E3" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3" s="20" t="s">
         <v>172</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>173</v>
       </c>
       <c r="G3" s="20" t="s">
         <v>12</v>
@@ -1702,16 +1724,16 @@
         <v>62</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D4" s="57" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" s="42" t="s">
+        <v>173</v>
+      </c>
+      <c r="F4" s="34" t="s">
         <v>174</v>
-      </c>
-      <c r="F4" s="34" t="s">
-        <v>175</v>
       </c>
       <c r="G4" s="20" t="s">
         <v>12</v>
@@ -1725,16 +1747,16 @@
         <v>63</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>186</v>
-      </c>
-      <c r="D5" s="57" t="s">
-        <v>68</v>
+        <v>185</v>
+      </c>
+      <c r="D5" s="71" t="s">
+        <v>226</v>
       </c>
       <c r="E5" s="43" t="s">
+        <v>175</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>176</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>177</v>
       </c>
       <c r="G5" s="20" t="s">
         <v>12</v>
@@ -1748,16 +1770,16 @@
         <v>64</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>188</v>
-      </c>
-      <c r="D6" s="57" t="s">
-        <v>68</v>
+        <v>187</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>224</v>
       </c>
       <c r="E6" s="43" t="s">
+        <v>177</v>
+      </c>
+      <c r="F6" s="24" t="s">
         <v>178</v>
-      </c>
-      <c r="F6" s="24" t="s">
-        <v>179</v>
       </c>
       <c r="G6" s="20" t="s">
         <v>12</v>
@@ -1771,16 +1793,16 @@
         <v>65</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D7" s="44" t="s">
-        <v>67</v>
+        <v>227</v>
       </c>
       <c r="E7" s="43" t="s">
+        <v>179</v>
+      </c>
+      <c r="F7" s="24" t="s">
         <v>180</v>
-      </c>
-      <c r="F7" s="24" t="s">
-        <v>181</v>
       </c>
       <c r="G7" s="20" t="s">
         <v>12</v>
@@ -1794,16 +1816,16 @@
         <v>29</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>66</v>
       </c>
       <c r="E8" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="F8" s="24" t="s">
         <v>182</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>183</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>12</v>
@@ -1969,9 +1991,9 @@
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.42578125" customWidth="1"/>
     <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" customWidth="1"/>
+    <col min="5" max="5" width="38.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="55.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="69.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" customWidth="1"/>
     <col min="9" max="9" width="22" bestFit="1" customWidth="1"/>
   </cols>
@@ -2018,13 +2040,13 @@
         <v>51</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G2" s="33" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>12</v>
@@ -2044,13 +2066,13 @@
         <v>52</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G3" s="33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>12</v>
@@ -2070,13 +2092,13 @@
         <v>17</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G4" s="37" t="s">
         <v>136</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="G4" s="37" t="s">
-        <v>137</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>12</v>
@@ -2096,13 +2118,13 @@
         <v>17</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G5" s="39" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>12</v>
@@ -2122,13 +2144,13 @@
         <v>17</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>12</v>
@@ -2148,13 +2170,13 @@
         <v>17</v>
       </c>
       <c r="E7" s="56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G7" s="46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>12</v>
@@ -2174,13 +2196,13 @@
         <v>17</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G8" s="32" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>12</v>
@@ -2191,7 +2213,7 @@
         <v>37</v>
       </c>
       <c r="B9" s="65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" s="64" t="s">
         <v>11</v>
@@ -2199,14 +2221,14 @@
       <c r="D9" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="48" t="s">
-        <v>142</v>
+      <c r="E9" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G9" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>12</v>
@@ -2217,7 +2239,7 @@
         <v>38</v>
       </c>
       <c r="B10" s="65" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" s="64" t="s">
         <v>11</v>
@@ -2226,13 +2248,13 @@
         <v>52</v>
       </c>
       <c r="E10" s="39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>12</v>
@@ -2243,7 +2265,7 @@
         <v>39</v>
       </c>
       <c r="B11" s="65" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" s="64" t="s">
         <v>11</v>
@@ -2252,13 +2274,13 @@
         <v>51</v>
       </c>
       <c r="E11" s="56" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G11" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>12</v>
@@ -2269,7 +2291,7 @@
         <v>40</v>
       </c>
       <c r="B12" s="65" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="64" t="s">
         <v>11</v>
@@ -2278,13 +2300,13 @@
         <v>51</v>
       </c>
       <c r="E12" s="48" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G12" s="39" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>12</v>
@@ -2295,7 +2317,7 @@
         <v>41</v>
       </c>
       <c r="B13" s="65" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C13" s="64" t="s">
         <v>11</v>
@@ -2304,13 +2326,13 @@
         <v>51</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>12</v>
@@ -2321,7 +2343,7 @@
         <v>42</v>
       </c>
       <c r="B14" s="65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C14" s="64" t="s">
         <v>11</v>
@@ -2330,13 +2352,13 @@
         <v>51</v>
       </c>
       <c r="E14" s="39" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>12</v>
@@ -2347,7 +2369,7 @@
         <v>43</v>
       </c>
       <c r="B15" s="65" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C15" s="64" t="s">
         <v>11</v>
@@ -2356,13 +2378,13 @@
         <v>13</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
@@ -2373,7 +2395,7 @@
         <v>44</v>
       </c>
       <c r="B16" s="65" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C16" s="64" t="s">
         <v>11</v>
@@ -2382,13 +2404,13 @@
         <v>13</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G16" s="39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>12</v>
@@ -2399,7 +2421,7 @@
         <v>45</v>
       </c>
       <c r="B17" s="65" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" s="64" t="s">
         <v>11</v>
@@ -2408,13 +2430,13 @@
         <v>13</v>
       </c>
       <c r="E17" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>12</v>
@@ -2425,7 +2447,7 @@
         <v>46</v>
       </c>
       <c r="B18" s="65" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C18" s="64" t="s">
         <v>11</v>
@@ -2434,13 +2456,13 @@
         <v>13</v>
       </c>
       <c r="E18" s="56" t="s">
-        <v>141</v>
+        <v>225</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G18" s="46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>12</v>
@@ -2448,25 +2470,25 @@
     </row>
     <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="65" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" s="65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C19" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G19" s="48" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>12</v>
@@ -2474,25 +2496,25 @@
     </row>
     <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="65" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B20" s="65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D20" s="65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G20" s="32" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>12</v>
@@ -2500,10 +2522,10 @@
     </row>
     <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B21" s="65" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C21" s="64" t="s">
         <v>11</v>
@@ -2511,14 +2533,14 @@
       <c r="D21" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="32" t="s">
-        <v>136</v>
+      <c r="E21" s="33" t="s">
+        <v>135</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H21" s="5" t="s">
         <v>12</v>
@@ -2526,51 +2548,51 @@
     </row>
     <row r="22" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="65" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B22" s="65" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C22" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D22" s="65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>209</v>
       </c>
       <c r="G22" s="39" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B23" s="65" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C23" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E23" s="56" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="G23" s="56" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>12</v>
@@ -2578,25 +2600,25 @@
     </row>
     <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C24" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D24" s="65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E24" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G24" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>12</v>
@@ -2604,25 +2626,25 @@
     </row>
     <row r="25" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B25" s="65" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C25" s="64" t="s">
         <v>11</v>
       </c>
       <c r="D25" s="65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>12</v>
@@ -2630,10 +2652,10 @@
     </row>
     <row r="26" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="65" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B26" s="65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C26" s="64" t="s">
         <v>11</v>
@@ -2642,13 +2664,13 @@
         <v>17</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G26" s="39" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>12</v>
@@ -2656,10 +2678,10 @@
     </row>
     <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="65" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B27" s="65" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C27" s="64" t="s">
         <v>11</v>
@@ -2668,13 +2690,13 @@
         <v>17</v>
       </c>
       <c r="E27" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>12</v>
@@ -2682,10 +2704,10 @@
     </row>
     <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="65" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B28" s="65" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C28" s="64" t="s">
         <v>11</v>
@@ -2694,13 +2716,13 @@
         <v>17</v>
       </c>
       <c r="E28" s="32" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G28" s="32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>12</v>
@@ -2711,7 +2733,7 @@
         <v>50</v>
       </c>
       <c r="B29" s="62" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C29" s="66" t="s">
         <v>15</v>
@@ -2720,13 +2742,13 @@
         <v>19</v>
       </c>
       <c r="E29" s="54" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F29" s="54" t="s">
+        <v>132</v>
+      </c>
+      <c r="G29" s="50" t="s">
         <v>133</v>
-      </c>
-      <c r="G29" s="50" t="s">
-        <v>134</v>
       </c>
       <c r="H29" s="61" t="s">
         <v>12</v>
@@ -2734,25 +2756,25 @@
     </row>
     <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="70" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B30" s="49" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C30" s="67" t="s">
         <v>15</v>
       </c>
       <c r="D30" s="68" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E30" s="53" t="s">
+        <v>129</v>
+      </c>
+      <c r="F30" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="53" t="s">
+      <c r="G30" s="53" t="s">
         <v>131</v>
-      </c>
-      <c r="G30" s="53" t="s">
-        <v>132</v>
       </c>
       <c r="H30" s="55" t="s">
         <v>12</v>
@@ -2760,25 +2782,25 @@
     </row>
     <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B31" s="49" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C31" s="67" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="68" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E31" s="53" t="s">
+        <v>126</v>
+      </c>
+      <c r="F31" s="51" t="s">
         <v>127</v>
       </c>
-      <c r="F31" s="51" t="s">
+      <c r="G31" s="53" t="s">
         <v>128</v>
-      </c>
-      <c r="G31" s="53" t="s">
-        <v>129</v>
       </c>
       <c r="H31" s="55" t="s">
         <v>12</v>
@@ -2786,10 +2808,10 @@
     </row>
     <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="70" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B32" s="63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="67" t="s">
         <v>15</v>
@@ -2798,13 +2820,13 @@
         <v>16</v>
       </c>
       <c r="E32" s="51" t="s">
+        <v>121</v>
+      </c>
+      <c r="F32" s="47" t="s">
         <v>122</v>
       </c>
-      <c r="F32" s="47" t="s">
+      <c r="G32" s="47" t="s">
         <v>123</v>
-      </c>
-      <c r="G32" s="47" t="s">
-        <v>124</v>
       </c>
       <c r="H32" s="55" t="s">
         <v>12</v>
@@ -2812,10 +2834,10 @@
     </row>
     <row r="33" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="70" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="63" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C33" s="67" t="s">
         <v>15</v>
@@ -2824,13 +2846,13 @@
         <v>52</v>
       </c>
       <c r="E33" s="51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F33" s="53" t="s">
+        <v>119</v>
+      </c>
+      <c r="G33" s="53" t="s">
         <v>120</v>
-      </c>
-      <c r="G33" s="53" t="s">
-        <v>121</v>
       </c>
       <c r="H33" s="55" t="s">
         <v>12</v>
@@ -2838,10 +2860,10 @@
     </row>
     <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="70" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B34" s="63" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C34" s="67" t="s">
         <v>15</v>
@@ -2850,13 +2872,13 @@
         <v>52</v>
       </c>
       <c r="E34" s="53" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F34" s="53" t="s">
+        <v>117</v>
+      </c>
+      <c r="G34" s="51" t="s">
         <v>118</v>
-      </c>
-      <c r="G34" s="51" t="s">
-        <v>119</v>
       </c>
       <c r="H34" s="55" t="s">
         <v>12</v>
@@ -2864,25 +2886,25 @@
     </row>
     <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="70" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B35" s="63" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C35" s="67" t="s">
         <v>15</v>
       </c>
       <c r="D35" s="68" t="s">
+        <v>112</v>
+      </c>
+      <c r="E35" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="E35" s="51" t="s">
-        <v>116</v>
-      </c>
-      <c r="F35" s="51" t="s">
+      <c r="G35" s="53" t="s">
         <v>114</v>
-      </c>
-      <c r="G35" s="53" t="s">
-        <v>115</v>
       </c>
       <c r="H35" s="55" t="s">
         <v>12</v>

</xml_diff>